<commit_message>
Economy v0.2: read maxLineHaulKm from config, add cargo allowedTiers
Replace the maxLineHaulKm Dart constant with settings.maxLineHaulKm.
Parse and validate cargo.allowedTiers, and make checkTripEligibility
reject cargo the vehicle cannot carry. Update CLAUDE.md design rules.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/economy_model.xlsx
+++ b/docs/economy_model.xlsx
@@ -153,7 +153,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="313">
   <si>
     <t xml:space="preserve">Vehicle Manager Bangladesh: economy model v0.1</t>
   </si>
@@ -356,6 +356,15 @@
     <t xml:space="preserve">Game value. Repair, cargo claim and downtime together.</t>
   </si>
   <si>
+    <t xml:space="preserve">Maximum line haul distance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">km</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design rule copied from Truck Manager: line hauls run terminal to terminal up to 400 km. Longer trips become contracts (post-MVP).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Toll per crossing (Tk, one way)</t>
   </si>
   <si>
@@ -410,7 +419,7 @@
     <t xml:space="preserve">Rate factor</t>
   </si>
   <si>
-    <t xml:space="preserve">Used by tiers</t>
+    <t xml:space="preserve">Allowed tiers (comma separated, no spaces)</t>
   </si>
   <si>
     <t xml:space="preserve">Reasoning</t>
@@ -419,7 +428,7 @@
     <t xml:space="preserve">Market goods</t>
   </si>
   <si>
-    <t xml:space="preserve">1-2</t>
+    <t xml:space="preserve">1,2</t>
   </si>
   <si>
     <t xml:space="preserve">Short bazaar runs.</t>
@@ -428,7 +437,7 @@
     <t xml:space="preserve">Parcels</t>
   </si>
   <si>
-    <t xml:space="preserve">2-5</t>
+    <t xml:space="preserve">2,3,4,5</t>
   </si>
   <si>
     <t xml:space="preserve">E-commerce pays a premium for speed and small lots.</t>
@@ -437,16 +446,16 @@
     <t xml:space="preserve">General dry</t>
   </si>
   <si>
-    <t xml:space="preserve">3-7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baseline. All fares are fitted to this.</t>
+    <t xml:space="preserve">3,4,5,6,7,11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baseline. Tier 11 included so prime movers can haul general freight in the MVP. All fares are fitted to this.</t>
   </si>
   <si>
     <t xml:space="preserve">Vegetables</t>
   </si>
   <si>
-    <t xml:space="preserve">3-6</t>
+    <t xml:space="preserve">3,4,5,6</t>
   </si>
   <si>
     <t xml:space="preserve">Perishable, from northern districts to Dhaka.</t>
@@ -455,7 +464,7 @@
     <t xml:space="preserve">Garments</t>
   </si>
   <si>
-    <t xml:space="preserve">5-7</t>
+    <t xml:space="preserve">5,6,7</t>
   </si>
   <si>
     <t xml:space="preserve">Export deadline at the port. Missing it costs a penalty (later feature).</t>
@@ -464,7 +473,7 @@
     <t xml:space="preserve">Rice</t>
   </si>
   <si>
-    <t xml:space="preserve">6-7</t>
+    <t xml:space="preserve">4,5,6,7</t>
   </si>
   <si>
     <t xml:space="preserve">Bulk, steady demand.</t>
@@ -473,7 +482,7 @@
     <t xml:space="preserve">Cement and rod</t>
   </si>
   <si>
-    <t xml:space="preserve">6, 9</t>
+    <t xml:space="preserve">6,9</t>
   </si>
   <si>
     <t xml:space="preserve">Heavy, low value per ton.</t>
@@ -2097,7 +2106,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -2434,6 +2443,20 @@
       </c>
       <c r="D25" s="12" t="s">
         <v>66</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B26" s="11" t="n">
+        <v>400</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -2464,7 +2487,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2474,7 +2497,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2492,27 +2515,27 @@
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B5" s="11" t="n">
         <v>0</v>
@@ -2532,7 +2555,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B6" s="11" t="n">
         <v>0</v>
@@ -2552,7 +2575,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B7" s="11" t="n">
         <v>0</v>
@@ -2572,7 +2595,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B8" s="11" t="n">
         <v>0</v>
@@ -2592,7 +2615,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B9" s="11" t="n">
         <v>0</v>
@@ -2612,7 +2635,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B10" s="11" t="n">
         <v>0</v>
@@ -2632,7 +2655,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B11" s="11" t="n">
         <v>0</v>
@@ -2678,7 +2701,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2692,184 +2715,184 @@
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B4" s="19" t="n">
         <v>1.2</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B5" s="19" t="n">
         <v>1.5</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B6" s="19" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B7" s="19" t="n">
         <v>1.2</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B8" s="19" t="n">
         <v>1.4</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B9" s="19" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B10" s="19" t="n">
         <v>0.9</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B11" s="19" t="n">
         <v>0.9</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B12" s="19" t="n">
         <v>2.2</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B13" s="19" t="n">
         <v>1.2</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B14" s="19" t="n">
         <v>1.2</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B15" s="19" t="n">
         <v>1.2</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -2913,7 +2936,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2937,7 +2960,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2983,64 +3006,64 @@
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="Q4" s="8" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="R4" s="8" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="S4" s="8" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="T4" s="8" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3048,10 +3071,10 @@
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D5" s="20" t="n">
         <v>0.2</v>
@@ -3092,13 +3115,13 @@
         <v>2.5</v>
       </c>
       <c r="P5" s="22" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="Q5" s="22" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="R5" s="22" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="S5" s="26" t="n">
         <v>0.5</v>
@@ -3112,10 +3135,10 @@
         <v>2</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D6" s="20" t="n">
         <v>1.5</v>
@@ -3156,13 +3179,13 @@
         <v>2.7</v>
       </c>
       <c r="P6" s="22" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="Q6" s="22" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="R6" s="22" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="S6" s="26" t="n">
         <v>1</v>
@@ -3176,10 +3199,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D7" s="20" t="n">
         <v>10</v>
@@ -3220,13 +3243,13 @@
         <v>3</v>
       </c>
       <c r="P7" s="22" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="Q7" s="22" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R7" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="S7" s="26" t="n">
         <v>5</v>
@@ -3240,10 +3263,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D8" s="20" t="n">
         <v>13</v>
@@ -3284,13 +3307,13 @@
         <v>2.8</v>
       </c>
       <c r="P8" s="22" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="Q8" s="22" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R8" s="22" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="S8" s="26" t="n">
         <v>5</v>
@@ -3304,10 +3327,10 @@
         <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D9" s="20" t="n">
         <v>25</v>
@@ -3348,13 +3371,13 @@
         <v>1.6</v>
       </c>
       <c r="P9" s="22" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="Q9" s="22" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R9" s="22" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="S9" s="26" t="n">
         <v>10</v>
@@ -3368,10 +3391,10 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D10" s="20" t="n">
         <v>32</v>
@@ -3412,13 +3435,13 @@
         <v>1</v>
       </c>
       <c r="P10" s="22" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="Q10" s="22" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R10" s="22" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="S10" s="26" t="n">
         <v>10</v>
@@ -3432,10 +3455,10 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="D11" s="20" t="n">
         <v>35</v>
@@ -3476,13 +3499,13 @@
         <v>1.05</v>
       </c>
       <c r="P11" s="22" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="Q11" s="22" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R11" s="22" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S11" s="26" t="n">
         <v>10</v>
@@ -3496,10 +3519,10 @@
         <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D12" s="20" t="n">
         <v>45</v>
@@ -3540,13 +3563,13 @@
         <v>1</v>
       </c>
       <c r="P12" s="22" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="Q12" s="22" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R12" s="22" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="S12" s="26" t="n">
         <v>10</v>
@@ -3560,10 +3583,10 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="D13" s="20" t="n">
         <v>60</v>
@@ -3604,13 +3627,13 @@
         <v>1.2</v>
       </c>
       <c r="P13" s="22" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="Q13" s="22" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R13" s="22" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="S13" s="26" t="n">
         <v>20</v>
@@ -3624,10 +3647,10 @@
         <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="D14" s="20" t="n">
         <v>50</v>
@@ -3668,13 +3691,13 @@
         <v>1</v>
       </c>
       <c r="P14" s="22" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="Q14" s="22" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R14" s="22" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="S14" s="26" t="n">
         <v>20</v>
@@ -3688,10 +3711,10 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D15" s="20" t="n">
         <v>65</v>
@@ -3732,13 +3755,13 @@
         <v>0.6</v>
       </c>
       <c r="P15" s="22" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="Q15" s="22" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R15" s="22" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="S15" s="26" t="n">
         <v>20</v>
@@ -3752,10 +3775,10 @@
         <v>12</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="D16" s="20" t="n">
         <v>80</v>
@@ -3796,13 +3819,13 @@
         <v>0.6</v>
       </c>
       <c r="P16" s="22" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="Q16" s="22" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R16" s="22" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="S16" s="26" t="n">
         <v>20</v>
@@ -3844,7 +3867,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3858,7 +3881,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3884,54 +3907,54 @@
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="D5" s="11" t="n">
         <v>3</v>
       </c>
       <c r="E5" s="22" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="F5" s="22" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G5" s="22" t="n">
         <v>0</v>
@@ -3943,27 +3966,27 @@
         <v>3</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="D6" s="11" t="n">
         <v>8</v>
       </c>
       <c r="E6" s="22" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="F6" s="22" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G6" s="22" t="n">
         <v>0</v>
@@ -3975,27 +3998,27 @@
         <v>8</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="D7" s="11" t="n">
         <v>15</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="F7" s="22" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G7" s="22" t="n">
         <v>0</v>
@@ -4007,27 +4030,27 @@
         <v>60</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D8" s="11" t="n">
         <v>20</v>
       </c>
       <c r="E8" s="22" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="F8" s="22" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G8" s="22" t="n">
         <v>0</v>
@@ -4042,22 +4065,22 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="D9" s="11" t="n">
         <v>35</v>
       </c>
       <c r="E9" s="22" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G9" s="22" t="n">
         <v>0</v>
@@ -4069,27 +4092,27 @@
         <v>80</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="D10" s="11" t="n">
         <v>100</v>
       </c>
       <c r="E10" s="22" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F10" s="22" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="G10" s="22" t="n">
         <v>1</v>
@@ -4104,22 +4127,22 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="D11" s="11" t="n">
         <v>250</v>
       </c>
       <c r="E11" s="22" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F11" s="22" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="G11" s="22" t="n">
         <v>2</v>
@@ -4131,27 +4154,27 @@
         <v>400</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="D12" s="11" t="n">
         <v>280</v>
       </c>
       <c r="E12" s="22" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F12" s="22" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="G12" s="22" t="n">
         <v>2</v>
@@ -4163,27 +4186,27 @@
         <v>300</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="D13" s="11" t="n">
         <v>240</v>
       </c>
       <c r="E13" s="22" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F13" s="22" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G13" s="22" t="n">
         <v>0</v>
@@ -4198,22 +4221,22 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="D14" s="11" t="n">
         <v>200</v>
       </c>
       <c r="E14" s="22" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F14" s="22" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="G14" s="22" t="n">
         <v>1</v>
@@ -4225,27 +4248,27 @@
         <v>150</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="D15" s="11" t="n">
         <v>300</v>
       </c>
       <c r="E15" s="22" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F15" s="22" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="G15" s="22" t="n">
         <v>1</v>
@@ -4260,22 +4283,22 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="D16" s="11" t="n">
         <v>220</v>
       </c>
       <c r="E16" s="22" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F16" s="22" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="G16" s="22" t="n">
         <v>0</v>
@@ -4287,27 +4310,27 @@
         <v>120</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="D17" s="11" t="n">
         <v>270</v>
       </c>
       <c r="E17" s="22" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F17" s="22" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="G17" s="22" t="n">
         <v>0</v>
@@ -4319,27 +4342,27 @@
         <v>120</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="D18" s="11" t="n">
         <v>200</v>
       </c>
       <c r="E18" s="22" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F18" s="22" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="G18" s="22" t="n">
         <v>0</v>
@@ -4351,27 +4374,27 @@
         <v>150</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="B19" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>212</v>
       </c>
       <c r="D19" s="11" t="n">
         <v>150</v>
       </c>
       <c r="E19" s="22" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F19" s="22" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G19" s="22" t="n">
         <v>1</v>
@@ -4386,22 +4409,22 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="D20" s="11" t="n">
         <v>25</v>
       </c>
       <c r="E20" s="22" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="F20" s="22" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G20" s="22" t="n">
         <v>0</v>
@@ -4413,7 +4436,7 @@
         <v>200</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
   </sheetData>
@@ -4464,7 +4487,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4500,7 +4523,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4570,82 +4593,82 @@
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="Q4" s="8" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="R4" s="8" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="S4" s="8" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="T4" s="8" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="U4" s="8" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="V4" s="8" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="W4" s="8" t="s">
         <v>14</v>
       </c>
       <c r="X4" s="8" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="Y4" s="8" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="Z4" s="8" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="AA4" s="8" t="s">
         <v>11</v>
@@ -4657,27 +4680,27 @@
         <v>13</v>
       </c>
       <c r="AD4" s="8" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="AE4" s="8" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="AF4" s="8" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B5" s="22" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="E5" s="23" t="n">
         <v>0</v>
@@ -4787,22 +4810,22 @@
         <v>0.4375</v>
       </c>
       <c r="AF5" s="5" t="str">
-        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B5,Vehicles!$A$5:$A$16,0))="No",K5="Line"),"Not allowed on highway","")</f>
+        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B5,Vehicles!$A$5:$A$16,0))="No",K5="Line"),"Not allowed on highway",IF(AND(K5="Line",L5&gt;Settings!$B$26),"Line haul too long",IF(ISERROR(SEARCH(","&amp;B5&amp;",",","&amp;INDEX(Cargo!$C$4:$C$15,MATCH($D5,Cargo!$A$4:$A$15,0))&amp;",")),"Cargo not allowed on this vehicle","")))</f>
         <v/>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="B6" s="22" t="n">
         <v>2</v>
       </c>
       <c r="C6" s="22" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="D6" s="22" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E6" s="23" t="n">
         <v>0</v>
@@ -4912,22 +4935,22 @@
         <v>0.866666666666667</v>
       </c>
       <c r="AF6" s="5" t="str">
-        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B6,Vehicles!$A$5:$A$16,0))="No",K6="Line"),"Not allowed on highway","")</f>
+        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B6,Vehicles!$A$5:$A$16,0))="No",K6="Line"),"Not allowed on highway",IF(AND(K6="Line",L6&gt;Settings!$B$26),"Line haul too long",IF(ISERROR(SEARCH(","&amp;B6&amp;",",","&amp;INDEX(Cargo!$C$4:$C$15,MATCH($D6,Cargo!$A$4:$A$15,0))&amp;",")),"Cargo not allowed on this vehicle","")))</f>
         <v/>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="B7" s="22" t="n">
         <v>3</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="D7" s="22" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E7" s="23" t="n">
         <v>0</v>
@@ -5037,22 +5060,22 @@
         <v>4.58333333333333</v>
       </c>
       <c r="AF7" s="5" t="str">
-        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B7,Vehicles!$A$5:$A$16,0))="No",K7="Line"),"Not allowed on highway","")</f>
+        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B7,Vehicles!$A$5:$A$16,0))="No",K7="Line"),"Not allowed on highway",IF(AND(K7="Line",L7&gt;Settings!$B$26),"Line haul too long",IF(ISERROR(SEARCH(","&amp;B7&amp;",",","&amp;INDEX(Cargo!$C$4:$C$15,MATCH($D7,Cargo!$A$4:$A$15,0))&amp;",")),"Cargo not allowed on this vehicle","")))</f>
         <v/>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="B8" s="22" t="n">
         <v>4</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="D8" s="22" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E8" s="23" t="n">
         <v>0</v>
@@ -5162,22 +5185,22 @@
         <v>2.33333333333333</v>
       </c>
       <c r="AF8" s="5" t="str">
-        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B8,Vehicles!$A$5:$A$16,0))="No",K8="Line"),"Not allowed on highway","")</f>
+        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B8,Vehicles!$A$5:$A$16,0))="No",K8="Line"),"Not allowed on highway",IF(AND(K8="Line",L8&gt;Settings!$B$26),"Line haul too long",IF(ISERROR(SEARCH(","&amp;B8&amp;",",","&amp;INDEX(Cargo!$C$4:$C$15,MATCH($D8,Cargo!$A$4:$A$15,0))&amp;",")),"Cargo not allowed on this vehicle","")))</f>
         <v/>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="B9" s="22" t="n">
         <v>5</v>
       </c>
       <c r="C9" s="22" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E9" s="23" t="n">
         <v>0</v>
@@ -5287,22 +5310,22 @@
         <v>4.65277777777778</v>
       </c>
       <c r="AF9" s="5" t="str">
-        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B9,Vehicles!$A$5:$A$16,0))="No",K9="Line"),"Not allowed on highway","")</f>
+        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B9,Vehicles!$A$5:$A$16,0))="No",K9="Line"),"Not allowed on highway",IF(AND(K9="Line",L9&gt;Settings!$B$26),"Line haul too long",IF(ISERROR(SEARCH(","&amp;B9&amp;",",","&amp;INDEX(Cargo!$C$4:$C$15,MATCH($D9,Cargo!$A$4:$A$15,0))&amp;",")),"Cargo not allowed on this vehicle","")))</f>
         <v/>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="B10" s="22" t="n">
         <v>6</v>
       </c>
       <c r="C10" s="22" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="D10" s="22" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E10" s="23" t="n">
         <v>0</v>
@@ -5412,22 +5435,22 @@
         <v>15.4166666666667</v>
       </c>
       <c r="AF10" s="5" t="str">
-        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B10,Vehicles!$A$5:$A$16,0))="No",K10="Line"),"Not allowed on highway","")</f>
+        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B10,Vehicles!$A$5:$A$16,0))="No",K10="Line"),"Not allowed on highway",IF(AND(K10="Line",L10&gt;Settings!$B$26),"Line haul too long",IF(ISERROR(SEARCH(","&amp;B10&amp;",",","&amp;INDEX(Cargo!$C$4:$C$15,MATCH($D10,Cargo!$A$4:$A$15,0))&amp;",")),"Cargo not allowed on this vehicle","")))</f>
         <v/>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="B11" s="22" t="n">
         <v>7</v>
       </c>
       <c r="C11" s="22" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="D11" s="22" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="E11" s="23" t="n">
         <v>0</v>
@@ -5537,22 +5560,22 @@
         <v>13.125</v>
       </c>
       <c r="AF11" s="5" t="str">
-        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B11,Vehicles!$A$5:$A$16,0))="No",K11="Line"),"Not allowed on highway","")</f>
+        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B11,Vehicles!$A$5:$A$16,0))="No",K11="Line"),"Not allowed on highway",IF(AND(K11="Line",L11&gt;Settings!$B$26),"Line haul too long",IF(ISERROR(SEARCH(","&amp;B11&amp;",",","&amp;INDEX(Cargo!$C$4:$C$15,MATCH($D11,Cargo!$A$4:$A$15,0))&amp;",")),"Cargo not allowed on this vehicle","")))</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="B12" s="22" t="n">
         <v>8</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="D12" s="22" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="E12" s="23" t="n">
         <v>0</v>
@@ -5662,22 +5685,22 @@
         <v>6.66666666666667</v>
       </c>
       <c r="AF12" s="5" t="str">
-        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B12,Vehicles!$A$5:$A$16,0))="No",K12="Line"),"Not allowed on highway","")</f>
+        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B12,Vehicles!$A$5:$A$16,0))="No",K12="Line"),"Not allowed on highway",IF(AND(K12="Line",L12&gt;Settings!$B$26),"Line haul too long",IF(ISERROR(SEARCH(","&amp;B12&amp;",",","&amp;INDEX(Cargo!$C$4:$C$15,MATCH($D12,Cargo!$A$4:$A$15,0))&amp;",")),"Cargo not allowed on this vehicle","")))</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="B13" s="22" t="n">
         <v>9</v>
       </c>
       <c r="C13" s="22" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="D13" s="22" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E13" s="23" t="n">
         <v>0</v>
@@ -5787,22 +5810,22 @@
         <v>1.69753086419753</v>
       </c>
       <c r="AF13" s="5" t="str">
-        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B13,Vehicles!$A$5:$A$16,0))="No",K13="Line"),"Not allowed on highway","")</f>
+        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B13,Vehicles!$A$5:$A$16,0))="No",K13="Line"),"Not allowed on highway",IF(AND(K13="Line",L13&gt;Settings!$B$26),"Line haul too long",IF(ISERROR(SEARCH(","&amp;B13&amp;",",","&amp;INDEX(Cargo!$C$4:$C$15,MATCH($D13,Cargo!$A$4:$A$15,0))&amp;",")),"Cargo not allowed on this vehicle","")))</f>
         <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="B14" s="22" t="n">
         <v>10</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="D14" s="22" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="E14" s="23" t="n">
         <v>0</v>
@@ -5912,22 +5935,22 @@
         <v>12.6050420168067</v>
       </c>
       <c r="AF14" s="5" t="str">
-        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B14,Vehicles!$A$5:$A$16,0))="No",K14="Line"),"Not allowed on highway","")</f>
+        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B14,Vehicles!$A$5:$A$16,0))="No",K14="Line"),"Not allowed on highway",IF(AND(K14="Line",L14&gt;Settings!$B$26),"Line haul too long",IF(ISERROR(SEARCH(","&amp;B14&amp;",",","&amp;INDEX(Cargo!$C$4:$C$15,MATCH($D14,Cargo!$A$4:$A$15,0))&amp;",")),"Cargo not allowed on this vehicle","")))</f>
         <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="B15" s="22" t="n">
         <v>11</v>
       </c>
       <c r="C15" s="22" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="D15" s="22" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E15" s="23" t="n">
         <v>0</v>
@@ -6037,22 +6060,22 @@
         <v>6.33503401360544</v>
       </c>
       <c r="AF15" s="5" t="str">
-        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B15,Vehicles!$A$5:$A$16,0))="No",K15="Line"),"Not allowed on highway","")</f>
+        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B15,Vehicles!$A$5:$A$16,0))="No",K15="Line"),"Not allowed on highway",IF(AND(K15="Line",L15&gt;Settings!$B$26),"Line haul too long",IF(ISERROR(SEARCH(","&amp;B15&amp;",",","&amp;INDEX(Cargo!$C$4:$C$15,MATCH($D15,Cargo!$A$4:$A$15,0))&amp;",")),"Cargo not allowed on this vehicle","")))</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="B16" s="22" t="n">
         <v>12</v>
       </c>
       <c r="C16" s="22" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="D16" s="22" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="E16" s="23" t="n">
         <v>0</v>
@@ -6162,22 +6185,22 @@
         <v>5.83333333333333</v>
       </c>
       <c r="AF16" s="5" t="str">
-        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B16,Vehicles!$A$5:$A$16,0))="No",K16="Line"),"Not allowed on highway","")</f>
+        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B16,Vehicles!$A$5:$A$16,0))="No",K16="Line"),"Not allowed on highway",IF(AND(K16="Line",L16&gt;Settings!$B$26),"Line haul too long",IF(ISERROR(SEARCH(","&amp;B16&amp;",",","&amp;INDEX(Cargo!$C$4:$C$15,MATCH($D16,Cargo!$A$4:$A$15,0))&amp;",")),"Cargo not allowed on this vehicle","")))</f>
         <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="B17" s="22" t="n">
         <v>6</v>
       </c>
       <c r="C17" s="22" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="D17" s="22" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E17" s="23" t="n">
         <v>0</v>
@@ -6287,22 +6310,22 @@
         <v>15.4166666666667</v>
       </c>
       <c r="AF17" s="5" t="str">
-        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B17,Vehicles!$A$5:$A$16,0))="No",K17="Line"),"Not allowed on highway","")</f>
+        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B17,Vehicles!$A$5:$A$16,0))="No",K17="Line"),"Not allowed on highway",IF(AND(K17="Line",L17&gt;Settings!$B$26),"Line haul too long",IF(ISERROR(SEARCH(","&amp;B17&amp;",",","&amp;INDEX(Cargo!$C$4:$C$15,MATCH($D17,Cargo!$A$4:$A$15,0))&amp;",")),"Cargo not allowed on this vehicle","")))</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="B18" s="22" t="n">
         <v>6</v>
       </c>
       <c r="C18" s="22" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="D18" s="22" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E18" s="23" t="n">
         <v>8</v>
@@ -6412,22 +6435,22 @@
         <v>8.56481481481481</v>
       </c>
       <c r="AF18" s="5" t="str">
-        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B18,Vehicles!$A$5:$A$16,0))="No",K18="Line"),"Not allowed on highway","")</f>
+        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B18,Vehicles!$A$5:$A$16,0))="No",K18="Line"),"Not allowed on highway",IF(AND(K18="Line",L18&gt;Settings!$B$26),"Line haul too long",IF(ISERROR(SEARCH(","&amp;B18&amp;",",","&amp;INDEX(Cargo!$C$4:$C$15,MATCH($D18,Cargo!$A$4:$A$15,0))&amp;",")),"Cargo not allowed on this vehicle","")))</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="B19" s="22" t="n">
         <v>6</v>
       </c>
       <c r="C19" s="22" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="D19" s="22" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E19" s="23" t="n">
         <v>12</v>
@@ -6537,22 +6560,22 @@
         <v>7.00757575757576</v>
       </c>
       <c r="AF19" s="5" t="str">
-        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B19,Vehicles!$A$5:$A$16,0))="No",K19="Line"),"Not allowed on highway","")</f>
+        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B19,Vehicles!$A$5:$A$16,0))="No",K19="Line"),"Not allowed on highway",IF(AND(K19="Line",L19&gt;Settings!$B$26),"Line haul too long",IF(ISERROR(SEARCH(","&amp;B19&amp;",",","&amp;INDEX(Cargo!$C$4:$C$15,MATCH($D19,Cargo!$A$4:$A$15,0))&amp;",")),"Cargo not allowed on this vehicle","")))</f>
         <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B20" s="22" t="n">
         <v>6</v>
       </c>
       <c r="C20" s="22" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="D20" s="22" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E20" s="23" t="n">
         <v>12</v>
@@ -6662,22 +6685,22 @@
         <v>1.60984848484848</v>
       </c>
       <c r="AF20" s="5" t="str">
-        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B20,Vehicles!$A$5:$A$16,0))="No",K20="Line"),"Not allowed on highway","")</f>
+        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B20,Vehicles!$A$5:$A$16,0))="No",K20="Line"),"Not allowed on highway",IF(AND(K20="Line",L20&gt;Settings!$B$26),"Line haul too long",IF(ISERROR(SEARCH(","&amp;B20&amp;",",","&amp;INDEX(Cargo!$C$4:$C$15,MATCH($D20,Cargo!$A$4:$A$15,0))&amp;",")),"Cargo not allowed on this vehicle","")))</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="B21" s="22" t="n">
         <v>6</v>
       </c>
       <c r="C21" s="22" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="D21" s="22" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E21" s="23" t="n">
         <v>0</v>
@@ -6787,22 +6810,22 @@
         <v>4</v>
       </c>
       <c r="AF21" s="5" t="str">
-        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B21,Vehicles!$A$5:$A$16,0))="No",K21="Line"),"Not allowed on highway","")</f>
+        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B21,Vehicles!$A$5:$A$16,0))="No",K21="Line"),"Not allowed on highway",IF(AND(K21="Line",L21&gt;Settings!$B$26),"Line haul too long",IF(ISERROR(SEARCH(","&amp;B21&amp;",",","&amp;INDEX(Cargo!$C$4:$C$15,MATCH($D21,Cargo!$A$4:$A$15,0))&amp;",")),"Cargo not allowed on this vehicle","")))</f>
         <v/>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="B22" s="22" t="n">
         <v>6</v>
       </c>
       <c r="C22" s="22" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="D22" s="22" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E22" s="23" t="n">
         <v>0</v>
@@ -6912,22 +6935,22 @@
         <v>7.375</v>
       </c>
       <c r="AF22" s="5" t="str">
-        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B22,Vehicles!$A$5:$A$16,0))="No",K22="Line"),"Not allowed on highway","")</f>
+        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B22,Vehicles!$A$5:$A$16,0))="No",K22="Line"),"Not allowed on highway",IF(AND(K22="Line",L22&gt;Settings!$B$26),"Line haul too long",IF(ISERROR(SEARCH(","&amp;B22&amp;",",","&amp;INDEX(Cargo!$C$4:$C$15,MATCH($D22,Cargo!$A$4:$A$15,0))&amp;",")),"Cargo not allowed on this vehicle","")))</f>
         <v/>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="B23" s="22" t="n">
         <v>4</v>
       </c>
       <c r="C23" s="22" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="D23" s="22" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E23" s="23" t="n">
         <v>0</v>
@@ -7037,22 +7060,22 @@
         <v>2.22222222222222</v>
       </c>
       <c r="AF23" s="5" t="str">
-        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B23,Vehicles!$A$5:$A$16,0))="No",K23="Line"),"Not allowed on highway","")</f>
+        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B23,Vehicles!$A$5:$A$16,0))="No",K23="Line"),"Not allowed on highway",IF(AND(K23="Line",L23&gt;Settings!$B$26),"Line haul too long",IF(ISERROR(SEARCH(","&amp;B23&amp;",",","&amp;INDEX(Cargo!$C$4:$C$15,MATCH($D23,Cargo!$A$4:$A$15,0))&amp;",")),"Cargo not allowed on this vehicle","")))</f>
         <v/>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B24" s="22" t="n">
         <v>5</v>
       </c>
       <c r="C24" s="22" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="D24" s="22" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E24" s="23" t="n">
         <v>0</v>
@@ -7162,22 +7185,22 @@
         <v>4.65277777777778</v>
       </c>
       <c r="AF24" s="5" t="str">
-        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B24,Vehicles!$A$5:$A$16,0))="No",K24="Line"),"Not allowed on highway","")</f>
+        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B24,Vehicles!$A$5:$A$16,0))="No",K24="Line"),"Not allowed on highway",IF(AND(K24="Line",L24&gt;Settings!$B$26),"Line haul too long",IF(ISERROR(SEARCH(","&amp;B24&amp;",",","&amp;INDEX(Cargo!$C$4:$C$15,MATCH($D24,Cargo!$A$4:$A$15,0))&amp;",")),"Cargo not allowed on this vehicle","")))</f>
         <v/>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="B25" s="22" t="n">
         <v>4</v>
       </c>
       <c r="C25" s="22" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="D25" s="22" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E25" s="23" t="n">
         <v>0</v>
@@ -7287,22 +7310,22 @@
         <v>5.33333333333333</v>
       </c>
       <c r="AF25" s="5" t="str">
-        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B25,Vehicles!$A$5:$A$16,0))="No",K25="Line"),"Not allowed on highway","")</f>
+        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B25,Vehicles!$A$5:$A$16,0))="No",K25="Line"),"Not allowed on highway",IF(AND(K25="Line",L25&gt;Settings!$B$26),"Line haul too long",IF(ISERROR(SEARCH(","&amp;B25&amp;",",","&amp;INDEX(Cargo!$C$4:$C$15,MATCH($D25,Cargo!$A$4:$A$15,0))&amp;",")),"Cargo not allowed on this vehicle","")))</f>
         <v/>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="B26" s="22" t="n">
         <v>1</v>
       </c>
       <c r="C26" s="22" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="D26" s="22" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E26" s="23" t="n">
         <v>0</v>
@@ -7412,7 +7435,7 @@
         <v>1808.33333333333</v>
       </c>
       <c r="AF26" s="5" t="str">
-        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B26,Vehicles!$A$5:$A$16,0))="No",K26="Line"),"Not allowed on highway","")</f>
+        <f aca="false">IF(AND(INDEX(Vehicles!$Q$5:$Q$16,MATCH($B26,Vehicles!$A$5:$A$16,0))="No",K26="Line"),"Not allowed on highway",IF(AND(K26="Line",L26&gt;Settings!$B$26),"Line haul too long",IF(ISERROR(SEARCH(","&amp;B26&amp;",",","&amp;INDEX(Cargo!$C$4:$C$15,MATCH($D26,Cargo!$A$4:$A$15,0))&amp;",")),"Cargo not allowed on this vehicle","")))</f>
         <v>Not allowed on highway</v>
       </c>
     </row>
@@ -7448,7 +7471,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -7461,7 +7484,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7485,7 +7508,7 @@
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="B4" s="7" t="n">
         <f aca="false">Settings!$B$16</f>
@@ -7495,7 +7518,7 @@
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="31" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="G4" s="5" t="n">
         <f aca="false">COUNTIFS($A$17:$A$65,"&lt;60",$F$17:$F$65,1)</f>
@@ -7506,7 +7529,7 @@
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="B5" s="7" t="n">
         <f aca="false">'Trip Calculator'!Z8</f>
@@ -7516,7 +7539,7 @@
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="31" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="G5" s="5" t="n">
         <f aca="false">SUM($F$17:$F$65)</f>
@@ -7532,7 +7555,7 @@
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="31" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="G6" s="21" t="n">
         <f aca="false">INDEX($H$17:$H$65,MATCH(Settings!$B$14,$A$17:$A$65,0))</f>
@@ -7543,16 +7566,16 @@
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
@@ -7565,7 +7588,7 @@
         <v>1</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="C8" s="7" t="n">
         <f aca="false">'Trip Calculator'!G7</f>
@@ -7586,7 +7609,7 @@
         <v>2</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="C9" s="7" t="n">
         <f aca="false">'Trip Calculator'!G23</f>
@@ -7607,7 +7630,7 @@
         <v>3</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="C10" s="7" t="n">
         <f aca="false">Settings!$B$17</f>
@@ -7627,7 +7650,7 @@
         <v>4</v>
       </c>
       <c r="B11" s="22" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="C11" s="7" t="n">
         <f aca="false">'Trip Calculator'!G25</f>
@@ -7648,7 +7671,7 @@
         <v>5</v>
       </c>
       <c r="B12" s="22" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="C12" s="7" t="n">
         <f aca="false">'Trip Calculator'!G24</f>
@@ -7669,7 +7692,7 @@
         <v>6</v>
       </c>
       <c r="B13" s="22" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="C13" s="7" t="n">
         <f aca="false">'Trip Calculator'!G10</f>
@@ -7709,31 +7732,31 @@
     </row>
     <row r="16" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="I16" s="8" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Limit Sonar Van to M routes and add a 6-slot garage cap
Economy config 0.3. Vehicles get allowedRoutes (tier 1: M01, M02; empty
means any route) and settings get startingGarageSlots = 6, counting the
free Sathi Plus. checkGarageSlot rejects a purchase with no free slot
(noFreeGarageSlot). Both are in the spreadsheet first (Vehicles column U,
Settings row 27), then economy.json. No existing balance number changed.

first_hours_sim.dart now honours the cap, adds policy D (highest profit per
hour) and reports cap minute, vehicles by tier, net worth. Policy A earns
less than D on every measure, so the cap works as intended. Cheap buyers
hit the cap in the first two minutes and sit on Tk 38 to 41 lakh by hour 3,
so slot expansion in Milestone 5 has to act as the cash sink.

PROJECT_STATUS.md updated (decisions, questions 1 and 4, R07 Bhairab toll
as a known gap).
</commit_message>
<xml_diff>
--- a/docs/economy_model.xlsx
+++ b/docs/economy_model.xlsx
@@ -2106,7 +2106,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -2457,6 +2457,26 @@
       </c>
       <c r="D26" s="12" t="s">
         <v>69</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Starting garage slots</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>vehicles</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>Game design value. Counts the free Sathi Plus, so the player can buy 5 more. A purchase with no free slot is rejected. Slot expansion comes with terminals (Milestone 5). Keeps cheap vehicles from compounding without limit during Turbo Start.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2911,7 +2931,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:T16"/>
+  <dimension ref="A1:U16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -2932,6 +2952,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="19" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="30"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3065,6 +3086,11 @@
       <c r="T4" s="8" t="s">
         <v>145</v>
       </c>
+      <c r="U4" s="8" t="inlineStr">
+        <is>
+          <t>Allowed routes (comma separated, no spaces, blank = any route)</t>
+        </is>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="n">
@@ -3129,6 +3155,11 @@
       <c r="T5" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="U5" s="22" t="inlineStr">
+        <is>
+          <t>M01,M02</t>
+        </is>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="n">
@@ -3193,6 +3224,7 @@
       <c r="T6" s="26" t="n">
         <v>10</v>
       </c>
+      <c r="U6" s="22"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="n">
@@ -3257,6 +3289,7 @@
       <c r="T7" s="26" t="n">
         <v>30</v>
       </c>
+      <c r="U7" s="22"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="n">
@@ -3321,6 +3354,7 @@
       <c r="T8" s="26" t="n">
         <v>30</v>
       </c>
+      <c r="U8" s="22"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="n">
@@ -3385,6 +3419,7 @@
       <c r="T9" s="26" t="n">
         <v>40</v>
       </c>
+      <c r="U9" s="22"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="n">
@@ -3449,6 +3484,7 @@
       <c r="T10" s="26" t="n">
         <v>40</v>
       </c>
+      <c r="U10" s="22"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="n">
@@ -3513,6 +3549,7 @@
       <c r="T11" s="26" t="n">
         <v>40</v>
       </c>
+      <c r="U11" s="22"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="n">
@@ -3577,6 +3614,7 @@
       <c r="T12" s="26" t="n">
         <v>40</v>
       </c>
+      <c r="U12" s="22"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="n">
@@ -3641,6 +3679,7 @@
       <c r="T13" s="26" t="n">
         <v>80</v>
       </c>
+      <c r="U13" s="22"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="n">
@@ -3705,6 +3744,7 @@
       <c r="T14" s="26" t="n">
         <v>80</v>
       </c>
+      <c r="U14" s="22"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="n">
@@ -3769,6 +3809,7 @@
       <c r="T15" s="26" t="n">
         <v>80</v>
       </c>
+      <c r="U15" s="22"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="n">
@@ -3833,6 +3874,7 @@
       <c r="T16" s="26" t="n">
         <v>80</v>
       </c>
+      <c r="U16" s="22"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Rename license to operating permit, add Company.permits, add policies F to H
Concept rename in the sheet (Operating Permits sheet, Vehicles column R
header, ids light, medium, heavy, coldchain, hazmat), economy.json
(permits, unlockPermit) and code (PermitSpec, checkPermitPurchase,
needsPermit). Permit prices are confirmed. No balance number changed.

Company.permits is a real field: unmodifiable set of ids, Hive adapter
field 5, optional, default empty. Old saves load with no permits and
committing a change keeps them. A permit purchase is not yet part of
ChangeSet; that comes with the buy screen.

first_hours_sim.dart: per-hour report, two idle-stretch measures, policy F
(E plus buying a permit that unlocks a better vehicle), and diagnostic
policies G and H (E and F with Line hauls). On Local routes F equals E
because the Dhaka Local routes are too small for permit-locked vehicles.
</commit_message>
<xml_diff>
--- a/docs/economy_model.xlsx
+++ b/docs/economy_model.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Tolls" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Cargo" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Vehicles" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Licenses" sheetId="9" state="visible" r:id="rId12"/>
+    <sheet name="Operating Permits" sheetId="9" state="visible" r:id="rId12"/>
     <sheet name="Routes" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="Trip Calculator" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="First Hour" sheetId="8" state="visible" r:id="rId10"/>
@@ -1724,7 +1724,7 @@
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Sheets: Settings (levers), Vehicles (12 tiers), Licenses (one-time Taka purchases that unlock tiers), Routes, Cargo, Tolls, Trip Calculator (one row per scenario), First Hour (purchase simulation).</t>
+          <t>Sheets: Settings (levers), Vehicles (12 tiers), Operating Permits (one-time Taka purchases that unlock tiers), Routes, Cargo, Tolls, Trip Calculator (one row per scenario), First Hour (purchase simulation).</t>
         </is>
       </c>
       <c r="B5" s="2"/>
@@ -3103,7 +3103,7 @@
       </c>
       <c r="R4" s="8" t="inlineStr">
         <is>
-          <t>Unlock: license id (blank = none, see Licenses sheet)</t>
+          <t>Unlock: operating permit id (blank = none, see Operating Permits sheet)</t>
         </is>
       </c>
       <c r="S4" s="8" t="s">
@@ -3657,7 +3657,7 @@
       </c>
       <c r="R12" s="22" t="inlineStr">
         <is>
-          <t>cold_chain</t>
+          <t>coldchain</t>
         </is>
       </c>
       <c r="S12" s="26" t="n">
@@ -9718,21 +9718,21 @@
     <row r="1" ht="17.35" customHeight="false">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Licenses</t>
+          <t>Operating permits</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>One-time Taka purchases. A vehicle with an unlock license id in the Vehicles sheet (column R) needs that license; tier 3 needs deliveries instead (column V).</t>
+          <t>One-time Taka purchases. A vehicle with an unlock permit id in the Vehicles sheet (column R) needs that permit; tier 3 needs deliveries instead (column V).</t>
         </is>
       </c>
     </row>
     <row r="3" ht="60" customHeight="true">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>License id</t>
+          <t>Permit id</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -9757,17 +9757,17 @@
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>License price as share of that vehicle's price</t>
+          <t>Permit price as share of that vehicle's price</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>Payback of that vehicle without the license (real h, typical route)</t>
+          <t>Payback of that vehicle without the permit (real h, typical route)</t>
         </is>
       </c>
       <c r="H3" s="8" t="inlineStr">
         <is>
-          <t>Payback with the license (real h)</t>
+          <t>Payback with the permit (real h)</t>
         </is>
       </c>
       <c r="I3" s="8" t="inlineStr">
@@ -9789,7 +9789,7 @@
       </c>
       <c r="B4" s="22" t="inlineStr">
         <is>
-          <t>Light license</t>
+          <t>Light operating permit</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
@@ -9821,7 +9821,7 @@
       </c>
       <c r="J4" s="12" t="inlineStr">
         <is>
-          <t>PROPOSED price: about 15 to 17 percent of the cheapest vehicle it unlocks. It adds about 2 to 5.5 real hours to that vehicle's payback at 1x (columns G and H, typical route) and keeps it inside its target range. One-time purchase in Taka, never a premium currency.</t>
+          <t>Confirmed price: about 15 to 17 percent of the cheapest vehicle it unlocks. It adds about 2 to 5.5 real hours to that vehicle's payback at 1x (columns G and H, typical route) and keeps it inside its target range. One-time purchase in Taka, never a premium currency.</t>
         </is>
       </c>
     </row>
@@ -9833,7 +9833,7 @@
       </c>
       <c r="B5" s="22" t="inlineStr">
         <is>
-          <t>Medium license</t>
+          <t>Medium operating permit</t>
         </is>
       </c>
       <c r="C5" s="15" t="n">
@@ -9872,12 +9872,12 @@
     <row r="6" ht="30" customHeight="true">
       <c r="A6" s="22" t="inlineStr">
         <is>
-          <t>cold_chain</t>
+          <t>coldchain</t>
         </is>
       </c>
       <c r="B6" s="22" t="inlineStr">
         <is>
-          <t>Cold chain license</t>
+          <t>Cold chain operating permit</t>
         </is>
       </c>
       <c r="C6" s="15" t="n">
@@ -9921,7 +9921,7 @@
       </c>
       <c r="B7" s="22" t="inlineStr">
         <is>
-          <t>Hazmat license</t>
+          <t>Hazmat operating permit</t>
         </is>
       </c>
       <c r="C7" s="15" t="n">
@@ -9965,7 +9965,7 @@
       </c>
       <c r="B8" s="22" t="inlineStr">
         <is>
-          <t>Heavy license</t>
+          <t>Heavy operating permit</t>
         </is>
       </c>
       <c r="C8" s="15" t="n">

</xml_diff>